<commit_message>
Auto update Pengadaan 2026-10-14 08:08:51
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-14).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-14).xlsx
@@ -1463,22 +1463,22 @@
         <v>1044316222</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>350117338</v>
+        <v>351115088</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>326386463</v>
+        <v>327384213</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>694198884</v>
+        <v>693201134</v>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1">
@@ -2119,10 +2119,10 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1153380061</v>
+        <v>1171480061</v>
       </c>
       <c r="E46" s="7" t="n">
         <v>10</v>
@@ -2137,10 +2137,10 @@
         <v>121983128</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>1028407160</v>
+        <v>1046507160</v>
       </c>
     </row>
     <row r="47" ht="45" customHeight="1">
@@ -3363,28 +3363,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3909</v>
+        <v>3910</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32965358267</v>
+        <v>32983458267</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6817694352</v>
+        <v>6818692102</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6376034170.6</v>
+        <v>6377031920.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>26147663915</v>
+        <v>26164766165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>